<commit_message>
Updated project issues excel
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAJARAMAN\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAJARAMAN\Desktop\Project Repo\microBank\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -106,12 +106,34 @@
     <t>To test document service for create bucket and file upload</t>
   </si>
   <si>
+    <t>To test document service connected to minio</t>
+  </si>
+  <si>
+    <t>Troubleshoot keycloak admin console https error when accessing from http other than localhost.
+Note: MUST USE ONLY FOR DEV OR TESTING AND NOT IN PROD</t>
+  </si>
+  <si>
+    <t>Use following parameters in docker-compose file.
+command:
+    -  start-dev
+    - --import-realm
+    - --hostname-strict=false
+    - --hostname-strict-https=false
+environment:
+KC_PROXY: edge
+KC_HTTP_ENABLED: "true"
+2. Edit the realm-export.json for sslRequired: "none" from "external"</t>
+  </si>
+  <si>
+    <t>VERY IMPORTANT: WHEN EDITING REALM.JSON FILE, MAKE SURE ANY EXISTING IMPORT INTO THE CONTAINER EXIST. OTHERWISE EVEN WHEN CHANGING JSON FILE NEW CHANGES MUST NOT TAKE EFFECT BECAUSE PREVIOUS VOLUME IS ATTACHED TO THE CONTAINER. THEREFORE IT IS IMPORTANT TO STOP AND REMOVE KEYCLOAK CONTAINER AND DELETE ANY NAMED VOLUME OR USE "docker compose down --volume"</t>
+  </si>
+  <si>
     <t>Step:1
 curl -X POST http://3.111.147.235:8123/api/v1/auth/login \
 -H "Content-Type: application/json" \
 -d '{
-        "username": "testuser",
-        "password": "Password123"
+        "username": "devops",
+        "password": "12345"
       }'
 Step:2
 api-gateway receives the above post request and forward to auth service which forwards to keycloak. Then keycloak verifies username/password and respond back with token, if valid, and in the below format.
@@ -125,28 +147,6 @@
 curl -X POST http://3.111.147.235:8123/api/v1/documents/upload \
 -H "Authorization: Bearer &lt;ACCESS_TOKEN&gt;" \
 -F "file=@test.pdf"</t>
-  </si>
-  <si>
-    <t>To test document service connected to minio</t>
-  </si>
-  <si>
-    <t>Troubleshoot keycloak admin console https error when accessing from http other than localhost.
-Note: MUST USE ONLY FOR DEV OR TESTING AND NOT IN PROD</t>
-  </si>
-  <si>
-    <t>Use following parameters in docker-compose file.
-command:
-    -  start-dev
-    - --import-realm
-    - --hostname-strict=false
-    - --hostname-strict-https=false
-environment:
-KC_PROXY: edge
-KC_HTTP_ENABLED: "true"
-2. Edit the realm-export.json for sslRequired: "none" from "external"</t>
-  </si>
-  <si>
-    <t>VERY IMPORTANT: WHEN EDITING REALM.JSON FILE, MAKE SURE ANY EXISTING IMPORT INTO THE CONTAINER EXIST. OTHERWISE EVEN WHEN CHANGING JSON FILE NEW CHANGES MUST NOT TAKE EFFECT BECAUSE PREVIOUS VOLUME IS ATTACHED TO THE CONTAINER. THEREFORE IT IS IMPORTANT TO STOP AND REMOVE KEYCLOAK CONTAINER AND DELETE ANY NAMED VOLUME OR USE "docker compose down --volume"</t>
   </si>
 </sst>
 </file>
@@ -610,13 +610,13 @@
         <v>6</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="315" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="330" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>7</v>
       </c>
@@ -624,7 +624,7 @@
         <v>25</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="225" x14ac:dyDescent="0.25">
@@ -632,13 +632,13 @@
         <v>8</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changing secret of keycloak client
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -125,12 +125,21 @@
 2. Edit the realm-export.json for sslRequired: "none" from "external"</t>
   </si>
   <si>
+    <t>curl -X POST http://&lt;HOST&gt;:9098/realms/microbank/protocol/openid-connect/token \
+-H "Content-Type: application/x-www-form-urlencoded" \
+-d "grant_type=password" \
+-d "client_id=microbank-client" \
+-d "client_secret=YOUR_SECRET" \
+-d "username=user1" \
+-d "password=user1"</t>
+  </si>
+  <si>
     <t>Step:1
 curl -X POST http://3.111.147.235:8123/api/v1/auth/login \
 -H "Content-Type: application/json" \
 -d '{
         "username": "devops",
-        "password": "12345"
+        "password": "devops"
       }'
 Step:2
 api-gateway receives the above post request and forward to auth service which forwards to keycloak. Then keycloak verifies username/password and respond back with token, if valid, and in the below format.
@@ -144,15 +153,6 @@
 curl -X POST http://3.111.147.235:8123/api/v1/documents/upload \
 -H "Authorization: Bearer &lt;ACCESS_TOKEN&gt;" \
 -F "file=@test.pdf"</t>
-  </si>
-  <si>
-    <t>curl -X POST http://&lt;HOST&gt;:9098/realms/microbank/protocol/openid-connect/token \
--H "Content-Type: application/x-www-form-urlencoded" \
--d "grant_type=password" \
--d "client_id=microbank-client" \
--d "client_secret=YOUR_SECRET" \
--d "username=user1" \
--d "password=user1"</t>
   </si>
 </sst>
 </file>
@@ -630,10 +630,10 @@
         <v>25</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="150" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updating api-gateway service app.yaml for auto service discovery
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -125,15 +125,6 @@
 2. Edit the realm-export.json for sslRequired: "none" from "external"</t>
   </si>
   <si>
-    <t>curl -X POST http://&lt;HOST&gt;:9098/realms/microbank/protocol/openid-connect/token \
--H "Content-Type: application/x-www-form-urlencoded" \
--d "grant_type=password" \
--d "client_id=microbank-client" \
--d "client_secret=YOUR_SECRET" \
--d "username=user1" \
--d "password=user1"</t>
-  </si>
-  <si>
     <t>Step:1
 curl -X POST http://3.111.147.235:8123/api/v1/auth/login \
 -H "Content-Type: application/json" \
@@ -153,6 +144,36 @@
 curl -X POST http://3.111.147.235:8123/api/v1/documents/upload \
 -H "Authorization: Bearer &lt;ACCESS_TOKEN&gt;" \
 -F "file=@test.pdf"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Bypassing auth service and validate client exist:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+curl -X POST http://&lt;HOST&gt;:9098/realms/microbank/protocol/openid-connect/token \
+-H "Content-Type: application/x-www-form-urlencoded" \
+-d "grant_type=password" \
+-d "client_id=microbank-client" \
+-d "client_secret=YOUR_SECRET" \
+-d "username=user1" \
+-d "password=user1"</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -630,10 +651,10 @@
         <v>25</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="150" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Documented keycloak issues in project excel file
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,10 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8340"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8340" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
+    <sheet name="keycloak" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -174,6 +175,56 @@
 -d "username=user1" \
 -d "password=user1"</t>
     </r>
+  </si>
+  <si>
+    <t>passed command parameters in docker compose as follows:
+"--hostname=keycloak", 
+"--hostname-port=8080"</t>
+  </si>
+  <si>
+    <t>Added new microbank-client user "devops" in keycloak through realm.json</t>
+  </si>
+  <si>
+    <t>issuer url mismatch:
+Springboot service issuer-uri points to keycloak:8080 but the keycloak issuer uri which is keycloak IP:PORT is 9098. i.e. container port is 8080 and host port is 9098.</t>
+  </si>
+  <si>
+    <t>Added devops user under "users" in realm-export.json</t>
+  </si>
+  <si>
+    <t>Microbank-client audience was not assigned, only account audience was existed, added protocol-mappers under clientId:"microbank-client" under clients</t>
+  </si>
+  <si>
+    <t>id: "a1b2c3d4-audience-microbank",
+"name": "audience microbank-client",
+  "protocol": "openid-connect",
+  "protocolMapper": "oidc-audience-mapper",
+  "consentRequired": false,
+  "config": {
+    "included.client.audience": "microbank-client",
+    "id.token.claim": "false",
+    "access.token.claim": "true"</t>
+  </si>
+  <si>
+    <t>id: "de0bb9e6-d0d5-41ea-8dcc-5e3a88d08df3",
+"name": "USER",
+"description": "",
+"composite": false,
+"clientRole": false,
+"containerId": "e48ddc52-5c93-4e3d-bc90-868d2332eb50",
+"attributes": {}</t>
+  </si>
+  <si>
+    <t>realmRoles: [
+"default-roles-microbank",
+      "USER"
+    ],</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application has @PreAuthorize("hasRole('USER')"), but the JWT payload does not contain "USER" role under realm access.
+1. Added "USER" role under realm under roles.
+2. Then assign this "USER" role to your user "devops" under realRoles. [SEE COMMENTS COLUMS]
+</t>
   </si>
 </sst>
 </file>
@@ -217,7 +268,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -230,6 +281,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -688,4 +742,83 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="69" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
+    <col min="5" max="10" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="135" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updating the project issues excel
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAJARAMAN\Desktop\Project Repo\microBank\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R RAJARAMAN\Desktop\Project Repo\microbank\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4D22BA-92C3-44D7-8693-CFD682CFFC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8340" activeTab="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
     <sheet name="keycloak" sheetId="2" r:id="rId2"/>
+    <sheet name="Minikube" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -226,11 +228,20 @@
 2. Then assign this "USER" role to your user "devops" under realRoles. [SEE COMMENTS COLUMS]
 </t>
   </si>
+  <si>
+    <t>By default, Images won't be available in minikube cluster. If it exist in dockerhub it will pulled or else you to explicitly have the built image in minikube cluster for testing</t>
+  </si>
+  <si>
+    <t>eval $(minikube docker-env)</t>
+  </si>
+  <si>
+    <t>run this command immediately after starting minikube cluster only then images built are avalable in minikube or else the built images will be on the host which is different docker-daemon.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -268,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -284,6 +295,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -564,17 +587,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="53.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="64.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="2"/>
+    <col min="2" max="2" width="53.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="64.109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -588,7 +611,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -602,7 +625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -619,7 +642,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -630,7 +653,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -644,12 +667,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -663,12 +686,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
@@ -676,17 +699,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C10" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>6</v>
       </c>
@@ -697,7 +720,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="330" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>7</v>
       </c>
@@ -711,7 +734,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="150" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>8</v>
       </c>
@@ -723,19 +746,19 @@
       </c>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D19" s="4"/>
     </row>
   </sheetData>
@@ -745,18 +768,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="1" max="1" width="9.109375" style="2"/>
     <col min="2" max="2" width="69" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
-    <col min="5" max="10" width="9.140625" style="2"/>
+    <col min="3" max="3" width="50.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="2" customWidth="1"/>
+    <col min="5" max="10" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -770,7 +793,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -781,7 +804,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -792,7 +815,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="135" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -803,7 +826,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="120" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -821,4 +844,54 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3816A58-5EAF-4E1F-A976-C2F368789B64}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="8"/>
+    <col min="2" max="2" width="47.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.21875" style="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adding k8s migration issues in excel
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R RAJARAMAN\Desktop\Project Repo\microbank\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RAJARAMAN\Desktop\Project Repo\microBank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4D22BA-92C3-44D7-8693-CFD682CFFC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
     <sheet name="keycloak" sheetId="2" r:id="rId2"/>
     <sheet name="Minikube" sheetId="3" r:id="rId3"/>
+    <sheet name="K8s Migration Issues" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="45">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -237,11 +237,17 @@
   <si>
     <t>run this command immediately after starting minikube cluster only then images built are avalable in minikube or else the built images will be on the host which is different docker-daemon.</t>
   </si>
+  <si>
+    <t>Removing service discovery results in feign client unable to find the k8s service DNS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add the service url in all feign client under account and transaction service </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -587,17 +593,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="2"/>
-    <col min="2" max="2" width="53.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="64.109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="53.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="64.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="32.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -611,7 +617,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -625,7 +631,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -642,7 +648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -653,7 +659,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -667,12 +673,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -686,12 +692,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C8" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C9" s="2" t="s">
         <v>20</v>
       </c>
@@ -699,17 +705,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C10" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>6</v>
       </c>
@@ -720,7 +726,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="330" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>7</v>
       </c>
@@ -734,7 +740,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="144" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>8</v>
       </c>
@@ -746,19 +752,19 @@
       </c>
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D19" s="4"/>
     </row>
   </sheetData>
@@ -768,18 +774,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="2"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="69" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="2" customWidth="1"/>
-    <col min="5" max="10" width="9.109375" style="2"/>
+    <col min="3" max="3" width="50.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
+    <col min="5" max="10" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
@@ -793,7 +799,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -804,7 +810,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -815,7 +821,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -826,7 +832,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -847,17 +853,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3816A58-5EAF-4E1F-A976-C2F368789B64}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="8"/>
-    <col min="2" max="2" width="47.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.44140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="47.21875" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="8"/>
+    <col min="2" max="2" width="47.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.28515625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>12</v>
       </c>
@@ -877,7 +883,7 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -889,6 +895,53 @@
       </c>
       <c r="D2" s="9" t="s">
         <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="8"/>
+    <col min="2" max="2" width="55.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated project and curl test
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="52">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -243,12 +243,46 @@
   <si>
     <t xml:space="preserve">Add the service url in all feign client under account and transaction service </t>
   </si>
+  <si>
+    <t>What you’ve accomplished already</t>
+  </si>
+  <si>
+    <t>Clean Kubernetes migration</t>
+  </si>
+  <si>
+    <t>Removed Eureka correctly</t>
+  </si>
+  <si>
+    <t>Fixed Feign clients</t>
+  </si>
+  <si>
+    <t>Solved DB DNS issues</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Switched to a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>proper local K8s platform</t>
+    </r>
+  </si>
+  <si>
+    <t>Set yourself up exactly like real platform teams do</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -259,6 +293,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -285,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -313,6 +355,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -904,7 +952,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="8"/>
@@ -944,6 +992,59 @@
         <v>44</v>
       </c>
     </row>
+    <row r="11" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="B11" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="11"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="11"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="11"/>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="11"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="11"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" s="11"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated curl test and project issue files
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -276,6 +276,37 @@
   </si>
   <si>
     <t>Set yourself up exactly like real platform teams do</t>
+  </si>
+  <si>
+    <t>nginx 404 error due to ingress not bound to api gateway</t>
+  </si>
+  <si>
+    <t>404 error via ingress from api gateway due to wait script at the entrypoint of
+ the api gateway service dockerfile</t>
+  </si>
+  <si>
+    <t>Removed wait script from dockerfile entrypoint rebuilt image and pushed to docker hub repository</t>
+  </si>
+  <si>
+    <t>502 bad gateway error due to tokens are generated via keycloak:80 which is a service DNS in kubernetes. But in application.yaml the token issuer validate from keycloak:8080 which is wrong.</t>
+  </si>
+  <si>
+    <t>Changed keycloak:8080 to keycloak. Port 80 is implicit no need to mention keycloak:80 (optional)</t>
+  </si>
+  <si>
+    <t>Added both annotation and ingress class name in ingress.yaml</t>
+  </si>
+  <si>
+    <t>Not a best practice to block one service from another service. K8s will take care of the readiness of the application at runtime using liveness and readiness probe.</t>
+  </si>
+  <si>
+    <t>DB not connected with application as application.yaml contains wrong hostname instead of k8s service DNS</t>
+  </si>
+  <si>
+    <t>Override service DNS in the env of the application deployment.</t>
+  </si>
+  <si>
+    <t>Best practice would be we may remove the DB connection config from application.yaml</t>
   </si>
 </sst>
 </file>
@@ -357,10 +388,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -956,9 +987,9 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="8"/>
-    <col min="2" max="2" width="55.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.140625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="56.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.42578125" style="9" customWidth="1"/>
     <col min="5" max="5" width="9.140625" style="8"/>
   </cols>
   <sheetData>
@@ -969,10 +1000,10 @@
       <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2"/>
@@ -981,7 +1012,7 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -990,6 +1021,56 @@
       </c>
       <c r="C2" s="9" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updating project issues file
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,13 +9,14 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
     <sheet name="keycloak" sheetId="2" r:id="rId2"/>
     <sheet name="Minikube" sheetId="3" r:id="rId3"/>
     <sheet name="K8s Migration Issues" sheetId="4" r:id="rId4"/>
+    <sheet name="CI" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="71">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -308,12 +309,54 @@
   <si>
     <t>Best practice would be we may remove the DB connection config from application.yaml</t>
   </si>
+  <si>
+    <t>Always keep CI file at the root of the project Directory</t>
+  </si>
+  <si>
+    <t>If in-case workflow file wrongly referenced, check the workflow context</t>
+  </si>
+  <si>
+    <t> - name: Show workflow execution context
+   run: |
+            echo "===== WORKFLOW DEBUG ====="
+            echo "Workflow file: $GITHUB_WORKFLOW"
+            echo "Repository: $GITHUB_REPOSITORY"
+            echo "Branch: $GITHUB_REF"
+            echo "Ref name: $GITHUB_REF_NAME"
+            echo "Commit SHA: $GITHUB_SHA"
+            echo "Actor: $GITHUB_ACTOR"
+            echo "=========================="</t>
+  </si>
+  <si>
+    <t>To get the workflow files use the following command</t>
+  </si>
+  <si>
+    <t>git ls-files | grep workflows</t>
+  </si>
+  <si>
+    <t>To delete/remove old workflow reference from git use this command</t>
+  </si>
+  <si>
+    <t>git rm -r --cached account/.github</t>
+  </si>
+  <si>
+    <t>To update version in gitops repo we have to mention the dev branch explicitly. Otherwise master branch is pointed by default</t>
+  </si>
+  <si>
+    <t> - name: Checkout GitOps repo
+   uses: actions/checkout@v4
+      with:
+        repository: Rajaraman-Ramanathan/microbank-gitops
+        ref: dev
+        token: ${{ secrets.GITOPS_PAT }}
+        path: microbank-gitops</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -337,6 +380,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -358,7 +406,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -392,6 +440,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1129,4 +1180,93 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="9"/>
+    <col min="2" max="2" width="49.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.140625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" style="9" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="150" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated project issues files
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="73">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -350,6 +350,14 @@
         ref: dev
         token: ${{ secrets.GITOPS_PAT }}
         path: microbank-gitops</t>
+  </si>
+  <si>
+    <t>To check whether gitops repo directory is correct, use this command</t>
+  </si>
+  <si>
+    <t> - name: Checkout GitOps repo
+    run: |
+        ls -R microbank-gitops</t>
   </si>
 </sst>
 </file>
@@ -406,7 +414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -441,7 +449,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1184,12 +1198,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="9"/>
     <col min="2" max="2" width="49.7109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.140625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="69.140625" style="13" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1200,7 +1214,7 @@
       <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="12" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="7" t="s">
@@ -1228,7 +1242,7 @@
       <c r="B3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="14" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1239,7 +1253,7 @@
       <c r="B4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="13" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1250,19 +1264,30 @@
       <c r="B5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="120" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="14" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated project issues file
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="4"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="80">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -358,6 +358,31 @@
     <t> - name: Checkout GitOps repo
     run: |
         ls -R microbank-gitops</t>
+  </si>
+  <si>
+    <t>Startup probe failed: Unable to connect to server port because server port removed from application.yaml and not added in k8s configmap. Therefore default tomcat port 8080 becomes the server port</t>
+  </si>
+  <si>
+    <t>Added server port on k8s configmap for all services and target the server port endpoint for health check.</t>
+  </si>
+  <si>
+    <t>.requestMatchers("/actuator/health/**").permitAll()
+.requestMatchers("/actuator/info").permitAll()</t>
+  </si>
+  <si>
+    <t>Startup probe failed 401 (Unauthorized): Actuator health endpoints should be explicitly permitted in security config of all services.</t>
+  </si>
+  <si>
+    <t>Startup probe failed 404: Actuator dependency missed in the pom.xml of notification service</t>
+  </si>
+  <si>
+    <t>&lt;dependency&gt;
+        &lt;groupId&gt;org.springframework.boot&lt;/groupId&gt;
+        &lt;artifactId&gt;spring-boot-starter-actuator&lt;/artifactId&gt;
+    &lt;/dependency&gt;</t>
+  </si>
+  <si>
+    <t>Added this dependency in notification service pom.xml</t>
   </si>
 </sst>
 </file>
@@ -414,7 +439,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -457,6 +482,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1138,6 +1166,42 @@
         <v>61</v>
       </c>
     </row>
+    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
     <row r="11" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
Updated curl and project issue files
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="3"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,8 @@
     <sheet name="Minikube" sheetId="3" r:id="rId3"/>
     <sheet name="K8s Migration Issues" sheetId="4" r:id="rId4"/>
     <sheet name="CI" sheetId="5" r:id="rId5"/>
+    <sheet name="argocd" sheetId="6" r:id="rId6"/>
+    <sheet name="helm" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="94">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -383,6 +385,50 @@
   </si>
   <si>
     <t>Added this dependency in notification service pom.xml</t>
+  </si>
+  <si>
+    <t>Always use following command when changing argocd manifest to sync</t>
+  </si>
+  <si>
+    <t>Argocd maintains an orphan resource policy so its very important to sync the apps manually If don't have argo UI</t>
+  </si>
+  <si>
+    <t>1. if changing in project - kubectl apply -f argocd/projects/platform-project.yaml
+2.  if changing in applications - kubectl apply -f argocd/applications/dev/keycloak.yaml
+3. Then annotate - kubectl annotate application keycloak-dev -n argocd argocd.argoproj.io/refresh=hard --overwrite</t>
+  </si>
+  <si>
+    <t>Always add repo first in your local</t>
+  </si>
+  <si>
+    <t>helm repo add bitnami https://charts.bitnami.com/bitnami</t>
+  </si>
+  <si>
+    <t>Then update repo</t>
+  </si>
+  <si>
+    <t>helm repo update</t>
+  </si>
+  <si>
+    <t>Use show command</t>
+  </si>
+  <si>
+    <t>helm show values bitnami/keycloak --version 24.3.0</t>
+  </si>
+  <si>
+    <t>docker search bitnami/keycloak</t>
+  </si>
+  <si>
+    <t>Use docker to search for chart under the repo</t>
+  </si>
+  <si>
+    <t>Use docker pull</t>
+  </si>
+  <si>
+    <t>docker pull bitnami/keycloak:25.0.0</t>
+  </si>
+  <si>
+    <t>Only after this validation add the registry, repo and tag all these 5 steps proves the reliability of available image and tags</t>
   </si>
 </sst>
 </file>
@@ -1358,4 +1404,147 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="65.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.5703125" style="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated project issue file
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" firstSheet="1" activeTab="5"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="98">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -393,42 +393,56 @@
     <t>Argocd maintains an orphan resource policy so its very important to sync the apps manually If don't have argo UI</t>
   </si>
   <si>
-    <t>1. if changing in project - kubectl apply -f argocd/projects/platform-project.yaml
-2.  if changing in applications - kubectl apply -f argocd/applications/dev/keycloak.yaml
+    <t>Always add repo first in your local</t>
+  </si>
+  <si>
+    <t>helm repo add bitnami https://charts.bitnami.com/bitnami</t>
+  </si>
+  <si>
+    <t>Then update repo</t>
+  </si>
+  <si>
+    <t>helm repo update</t>
+  </si>
+  <si>
+    <t>Use show command</t>
+  </si>
+  <si>
+    <t>helm show values bitnami/keycloak --version 24.3.0</t>
+  </si>
+  <si>
+    <t>docker search bitnami/keycloak</t>
+  </si>
+  <si>
+    <t>Use docker to search for chart under the repo</t>
+  </si>
+  <si>
+    <t>Use docker pull</t>
+  </si>
+  <si>
+    <t>docker pull bitnami/keycloak:25.0.0</t>
+  </si>
+  <si>
+    <t>Only after this validation add the registry, repo and tag all these 5 steps proves the reliability of available image and tags</t>
+  </si>
+  <si>
+    <t>For wrapper chart,i.e. Chart.yaml has dependency name then this name influence the values file. Example: postgress-wrapper becomes root chart, dependency name postgresql becomes dependency chart. Therefore in values file the root level definition will be name of the dependency chart and in this case its "postgresql"</t>
+  </si>
+  <si>
+    <t>Always move to chart folder and execute following commands:
+1. helm dependency build - This creates chart.lock and chart folder
+2. helm template test . -f values-dev.yaml - This command outputs the k8s template with values applied.</t>
+  </si>
+  <si>
+    <t>1. if changes in project - kubectl apply -f argocd/projects/platform-project.yaml
+2.  if changes in applications - kubectl apply -f argocd/applications/dev/keycloak.yaml
 3. Then annotate - kubectl annotate application keycloak-dev -n argocd argocd.argoproj.io/refresh=hard --overwrite</t>
   </si>
   <si>
-    <t>Always add repo first in your local</t>
-  </si>
-  <si>
-    <t>helm repo add bitnami https://charts.bitnami.com/bitnami</t>
-  </si>
-  <si>
-    <t>Then update repo</t>
-  </si>
-  <si>
-    <t>helm repo update</t>
-  </si>
-  <si>
-    <t>Use show command</t>
-  </si>
-  <si>
-    <t>helm show values bitnami/keycloak --version 24.3.0</t>
-  </si>
-  <si>
-    <t>docker search bitnami/keycloak</t>
-  </si>
-  <si>
-    <t>Use docker to search for chart under the repo</t>
-  </si>
-  <si>
-    <t>Use docker pull</t>
-  </si>
-  <si>
-    <t>docker pull bitnami/keycloak:25.0.0</t>
-  </si>
-  <si>
-    <t>Only after this validation add the registry, repo and tag all these 5 steps proves the reliability of available image and tags</t>
+    <t xml:space="preserve">Important:  charts folder should be moved to artifact registries such as jfrog or harbor </t>
+  </si>
+  <si>
+    <t>Always do template test before actual rollout</t>
   </si>
 </sst>
 </file>
@@ -485,7 +499,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -530,6 +544,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1445,7 +1462,7 @@
         <v>80</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
         <v>81</v>
@@ -1458,12 +1475,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="31.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="50.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="8"/>
+    <col min="2" max="2" width="43.5703125" style="15" customWidth="1"/>
+    <col min="3" max="3" width="64" style="8" customWidth="1"/>
+    <col min="4" max="4" width="50.5703125" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1487,64 +1505,84 @@
       <c r="J1" s="2"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>2</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C3" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C4" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D6" s="15" t="s">
+    </row>
+    <row r="7" spans="1:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>93</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="16" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added kind cluster config steps file and updated project issues file
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="2"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="123">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -536,6 +536,12 @@
   </si>
   <si>
     <t>For dns rewrite in kind cluster use edit command on coredns configmap</t>
+  </si>
+  <si>
+    <t>If issue like ip 127.0.0.1 in kube config then need to change correct ip address of dev cluster control plane.</t>
+  </si>
+  <si>
+    <t>kubectl config set-cluster kind-microbank-dev --server=https://172.18.0.4:6443</t>
   </si>
 </sst>
 </file>
@@ -1562,13 +1568,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="8" customWidth="1"/>
     <col min="2" max="2" width="65.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="72.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.28515625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1601,7 +1607,7 @@
       <c r="C2" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="9" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1614,6 +1620,17 @@
       </c>
       <c r="C3" s="9" t="s">
         <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated project issues file and proj arch
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" activeTab="5"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="docker-compose" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="137">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -515,18 +515,6 @@
 kubectl apply -f https://github.com/kubernetes-sigs/metrics-server/releases/latest/download/components.yaml</t>
   </si>
   <si>
-    <t>To avoid cpu, memory, sync issues do the following in argocd:
-1. Increase argocd timeout
-2. Reduce parallelism in argocd</t>
-  </si>
-  <si>
-    <t>1.kubectl edit configmap argocd-cm -n argocd
-2. Add the following
-    data:
-        timeout.reconciliation: 300s
-        application.controller.parallelism.limit: "2"</t>
-  </si>
-  <si>
     <t>rewrite name auth.microbank.local keycloak.keycloak.svc.cluster.local
 kubernetes cluster.local in-addr.arpa ip6.arpa {
        pods insecure
@@ -542,6 +530,88 @@
   </si>
   <si>
     <t>kubectl config set-cluster kind-microbank-dev --server=https://172.18.0.4:6443</t>
+  </si>
+  <si>
+    <t>Argocd applications and projects should run only in arogcd hub cluster. Only in this cluster we are running argocd CRD.</t>
+  </si>
+  <si>
+    <t>There your root argocd app destination server should always be argocd cluster and not dev or prod clusters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To avoid cpu, memory, sync issues do the following in argocd:
+1. Increase argocd timeout
+</t>
+  </si>
+  <si>
+    <t>1.kubectl edit configmap argocd-cm -n argocd
+2. Add the following
+    data:
+        timeout.reconciliation: 300s
+3. kubectl rollout restart deployment argocd-repo-server -n argocd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To avoid cpu, memory, sync issues do the following in argocd:
+1.Tune repo server resource request and limit
+</t>
+  </si>
+  <si>
+    <t>1. kubectl edit deployment argocd-repo-server -n argocd
+2. Add the following
+    resources:
+            requests:
+              memory: 512Mi
+              cpu: 250m
+            limits:
+              memory: 1Gi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To avoid cpu, memory, sync issues do the following in argocd:
+1.Update controller processors in configmap
+</t>
+  </si>
+  <si>
+    <t>1. kubectl edit configmap argocd-cmd-params-cm -n argocd
+2. Add the following
+    data:
+      application.controller.operation.processors: "2" # Controls parallel app sync
+      application.controller.status.processors: "2"  # limits reconciliation load
+3. kubectl rollout restart statefulset argocd-application-controller -n argocd</t>
+  </si>
+  <si>
+    <t>Verify step 2, 3, 4 use following command</t>
+  </si>
+  <si>
+    <t>kubectl logs -n argocd deploy/argocd-application-controller -f
+we should see following output.
+Processing app X
+Processing app Y
+(waiting… no more than 2 at once)</t>
+  </si>
+  <si>
+    <t>kubectl get all -n postgres -o json | \
+jq '.items[] | select(.metadata.finalizers!=null) | .metadata.name' -r | \
+xargs -I {} kubectl patch {} -n postgres -p '{"metadata":{"finalizers":[]}}' --type=merge</t>
+  </si>
+  <si>
+    <t>To remove namespace stuck in terminating state. But this require jquery installed.</t>
+  </si>
+  <si>
+    <t>To remove namespace stuck in terminating state. Emptying finalizer of specific resource such postgres-init-job in this case.</t>
+  </si>
+  <si>
+    <t>1. kubectl get all -n postgres -o json | grep finalizers -n
+2.kubectl patch job postgres-init-job -n postgres \
+    -p '{"metadata":{"finalizers":[]}}' \
+    --type=merge</t>
+  </si>
+  <si>
+    <t>Common culprits for namespace stuck in termination state</t>
+  </si>
+  <si>
+    <t>Jobs / Pods
+CRDs (ArgoCD apps, etc.)
+PVCs
+Finalizers not removed</t>
   </si>
 </sst>
 </file>
@@ -1233,10 +1303,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1568,12 +1638,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="65.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="72.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="65.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.42578125" style="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="42.28515625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1601,7 +1671,7 @@
       <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>80</v>
       </c>
       <c r="C2" s="9" t="s">
@@ -1616,21 +1686,98 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
+        <v>5</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>7</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>8</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>9</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added various integration plan documents
</commit_message>
<xml_diff>
--- a/project_issues.xlsx
+++ b/project_issues.xlsx
@@ -19,6 +19,7 @@
     <sheet name="CI" sheetId="5" r:id="rId5"/>
     <sheet name="argocd" sheetId="6" r:id="rId6"/>
     <sheet name="helm" sheetId="7" r:id="rId7"/>
+    <sheet name="Istio" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="163">
   <si>
     <t>docker exec -it api-gateway ping keycloak</t>
   </si>
@@ -670,6 +671,63 @@
   </si>
   <si>
     <t>Most important in ingress setup is to make hostport 80 and 443 to false. Because enabling this would make ingress container binds directly to nodePort network interface which violate security best practices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Istio base chart </t>
+  </si>
+  <si>
+    <t>helm repo add istio https://istio-release.storage.googleapis.com/charts
+helm pull istio/base \
+  --version 1.26.0 \
+  --untar \
+  --untardir charts</t>
+  </si>
+  <si>
+    <t>helm pull istio/cni \
+--version 1.26.0 \
+  --untar \
+  --untardir charts</t>
+  </si>
+  <si>
+    <t>Istio cni chart</t>
+  </si>
+  <si>
+    <t>helm pull istio/istiod \
+--version 1.26.0 \
+  --untar \
+  --untardir charts</t>
+  </si>
+  <si>
+    <t>Istiod chart</t>
+  </si>
+  <si>
+    <t>helm pull istio/gateway \
+--version 1.26.0 \
+  --untar \
+  --untardir charts</t>
+  </si>
+  <si>
+    <t>ingress gateway</t>
+  </si>
+  <si>
+    <t>Helm validations before actually apply</t>
+  </si>
+  <si>
+    <t>1. helm template auth-service  . -f test-values.yaml --debug
+2. helm template auth-service . -f test-values.yaml &gt; output.yaml
+3. helm lint .
+4. kubectl apply -f output.yaml --dry-run=client
+5. Enterprise validation using kubeconform: teams use this in CI
+helm template auth-service . | kubeconform -strict
+6. simulate install:
+This will catches missing values, template errors, include errors, indentation errors.
+helm install auth-service . --dry-run --debug</t>
+  </si>
+  <si>
+    <t>Helm template with actual dev values file.</t>
+  </si>
+  <si>
+    <t>helm template &lt;service-name&gt; ./charts/microservice-base -f ./&lt;service&gt;/values-dev.yaml</t>
   </si>
 </sst>
 </file>
@@ -1895,12 +1953,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="8"/>
     <col min="2" max="2" width="43.5703125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="64" style="8" customWidth="1"/>
+    <col min="3" max="3" width="82.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="50.5703125" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2071,23 +2129,45 @@
         <v>136</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="7" t="s">
+    <row r="14" spans="1:10" ht="150" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <v>13</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" s="7" t="s">
         <v>106</v>
       </c>
     </row>
@@ -2095,4 +2175,77 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="66.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>157</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>